<commit_message>
version for photochem comparison
</commit_message>
<xml_diff>
--- a/hu-code-sr/Documentation/SpeciesName.xlsx
+++ b/hu-code-sr/Documentation/SpeciesName.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11013"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sukrit/Documents/Research_Code/Hu_Code/hu-code-git/hu-code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailarizona-my.sharepoint.com/personal/wangjingyu_arizona_edu/Documents/Documents/PhD_Research/MEAC/updates-to-meac/Documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F8C30F-683D-1D4D-AEE2-756BE9E150FC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{34F8C30F-683D-1D4D-AEE2-756BE9E150FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{726E6201-D17E-AA41-82B6-3E7179F06A79}"/>
   <bookViews>
     <workbookView xWindow="3140" yWindow="2520" windowWidth="10000" windowHeight="11960" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -224,10 +224,6 @@
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
   <si>
-    <t>HSO2</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
     <t>OCS</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -454,6 +450,9 @@
   <si>
     <t>S8A</t>
     <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>HOSO</t>
   </si>
 </sst>
 </file>
@@ -1246,7 +1245,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>49</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1254,7 +1253,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1262,7 +1261,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1270,7 +1269,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1278,7 +1277,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1286,7 +1285,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1294,7 +1293,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1302,7 +1301,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1310,7 +1309,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1318,7 +1317,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1326,7 +1325,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1334,7 +1333,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1342,7 +1341,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1350,7 +1349,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1358,7 +1357,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1366,7 +1365,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1374,7 +1373,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1382,7 +1381,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1390,7 +1389,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1398,7 +1397,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1406,7 +1405,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1414,7 +1413,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1422,7 +1421,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1430,7 +1429,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1438,7 +1437,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1446,7 +1445,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1454,7 +1453,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1462,7 +1461,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1470,7 +1469,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1478,7 +1477,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1486,7 +1485,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1494,7 +1493,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1502,7 +1501,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1510,7 +1509,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1518,7 +1517,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1526,7 +1525,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1534,7 +1533,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1542,7 +1541,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1550,7 +1549,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1558,7 +1557,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1566,7 +1565,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1574,7 +1573,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1582,7 +1581,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1590,7 +1589,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1598,7 +1597,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1606,7 +1605,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1614,7 +1613,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1622,7 +1621,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1630,7 +1629,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1638,7 +1637,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1646,7 +1645,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1654,7 +1653,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1662,7 +1661,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1670,7 +1669,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1678,7 +1677,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1686,7 +1685,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1694,7 +1693,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1702,7 +1701,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1710,7 +1709,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1718,7 +1717,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1726,7 +1725,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1734,7 +1733,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1742,7 +1741,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="17" x14ac:dyDescent="0.2">
@@ -1750,7 +1749,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>